<commit_message>
modifications to simplified cases
</commit_message>
<xml_diff>
--- a/data/carriers_data/biomass/biomass_availability.xlsx
+++ b/data/carriers_data/biomass/biomass_availability.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\data\carriers_data\biomass\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164D22CA-BB0C-466D-94FF-9F5CC1D43DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCEEDF2-60D0-417B-A932-0E110E15F8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2400" yWindow="-14100" windowWidth="21600" windowHeight="11235" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Note" sheetId="4" r:id="rId1"/>
@@ -50,7 +50,7 @@
     <t>DE</t>
   </si>
   <si>
-    <t>Availability is expressed in PJ</t>
+    <t>Availability is expressed in PJ/y</t>
   </si>
 </sst>
 </file>

</xml_diff>